<commit_message>
Uniformização e renomear colunas
</commit_message>
<xml_diff>
--- a/output/Compared_2025-08-14.xlsx
+++ b/output/Compared_2025-08-14.xlsx
@@ -431,42 +431,42 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ean</t>
+          <t>Código de barras</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>Curva</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>best_external_price</t>
+          <t>Preço concorrente</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>best_external</t>
+          <t>Melhor concorrente</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>best</t>
+          <t>Comparação</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>internal_price</t>
+          <t>Preço oferta</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>Nome</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>external_url</t>
+          <t>Link concorrente</t>
         </is>
       </c>
     </row>

</xml_diff>